<commit_message>
Close out Sprint 4 story PRO-001
Records ADR-016 (the new provider -> identity role-grant direction,
reversing ADR-014), documents the temporary providers.category_label
column, backfills the still-missing Maps/Geocoding packages from
CUS-002 into the approved package list, updates project state and the
tracker to mark PRO-001 done, and adds the story's Walkthrough.
Removes the interim Checkpoint doc now that its content is folded
into the Walkthrough.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -9963,7 +9963,7 @@
       <c r="K26" s="10"/>
       <c r="L26" s="10"/>
       <c r="M26" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N26" s="10"/>
       <c r="O26" s="10" t="s">
@@ -9971,7 +9971,7 @@
       </c>
       <c r="P26" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M26)),1,IF(ISNUMBER(SEARCH("In Progress",M26)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="66" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Close out Sprint 4 story PRO-002 and complete Sprint 4
Records ADR-017 (the new FileStorage/LocalFileStorage abstraction,
this codebase's first file-upload capability), documents the four
new provider-storefront tables including the temporary
provider_category_labels table and the drop of providers.category_label,
backfills image_picker and python-multipart into the approved package
lists, adds the story's Walkthrough, and updates project state and
the tracker to mark PRO-002 done and Sprint 4 (Provider Storefront)
fully complete.

Verified VER-001 (Sprint 5) depends only on PRO-001, not PRO-002, so
it was already unblocked -- confirmed directly from the tracker
rather than left as a hedge.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4370,7 +4370,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.28958333333333336</v>
+        <v>0.31666666666666665</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4389,7 +4389,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4421,7 +4421,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">'Phase Tracker'!E3</f>
-        <v>0.2916666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="I9" s="0" t="s">
         <v>25</v>
@@ -4445,7 +4445,7 @@
         <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
@@ -4461,7 +4461,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,7 +4493,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">COUNTA(Milestones!$B$2:$B$25)</f>
@@ -4517,7 +4517,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4541,7 +4541,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -4590,7 +4590,7 @@
         <v>36</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B7</f>
-        <v>0.28958333333333336</v>
+        <v>0.31666666666666665</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
@@ -5388,7 +5388,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.2916666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5725,11 +5725,11 @@
       <c r="I5" s="12"/>
       <c r="J5" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B5)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B5),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K5" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B5,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J5=1,"✅ Completed",IF(J5&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="L5" s="12" t="n">
         <v>0</v>
@@ -6572,11 +6572,11 @@
       <c r="I7" s="10"/>
       <c r="J7" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C7)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C7),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K7" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C7,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J7=1,"✅ Completed",IF(J7&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7792,15 +7792,15 @@
       </c>
       <c r="H5" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A5)*(Stories!$P$2:$P$200))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I5" s="11" t="n">
         <f aca="false">IFERROR(H5/G5,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J5" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A5,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I5=1,"✅ Completed",IF(I5&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="K5" s="10" t="s">
         <v>72</v>
@@ -10006,7 +10006,7 @@
       <c r="K27" s="10"/>
       <c r="L27" s="10"/>
       <c r="M27" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N27" s="10"/>
       <c r="O27" s="10" t="s">
@@ -10014,7 +10014,7 @@
       </c>
       <c r="P27" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M27)),1,IF(ISNUMBER(SEARCH("In Progress",M27)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="78.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Sync Project_Tracker.xlsx: VER-001 done, Sprint 5 in progress
Marks VER-001 Done and refreshes every formula-driven rollup that
reads from it (Sprints, Milestones, Epics, Phase Tracker, Dashboard):
Sprint 5 and Milestone ML5 now show In Progress (1 of 2 stories
done), Epic ML5-EP01 (VER-001's own epic) shows Completed since it
has no other stories, and the Dashboard's completed-epic/story counts
and overall progress percentage are current. Applied via the same
raw-XML cell patching used for prior syncs, to avoid the
conditional-formatting-dropping issue an openpyxl round-trip causes
on this workbook.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4370,7 +4370,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.31666666666666665</v>
+        <v>0.34375</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4389,7 +4389,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4461,7 +4461,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4517,7 +4517,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4541,7 +4541,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B7</f>
-        <v>0.31666666666666665</v>
+        <v>0.34375</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
@@ -5388,7 +5388,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.3333333333333333</v>
+        <v>0.375</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5757,11 +5757,11 @@
       <c r="I6" s="12"/>
       <c r="J6" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B6)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B6),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K6" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B6,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J6=1,"✅ Completed",IF(J6&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="L6" s="12" t="n">
         <v>0</v>
@@ -6601,11 +6601,11 @@
       <c r="I8" s="10"/>
       <c r="J8" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C8)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C8),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K8" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C8,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J8=1,"✅ Completed",IF(J8&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7831,15 +7831,15 @@
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A6)*(Stories!$P$2:$P$200))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" s="11" t="n">
         <f aca="false">IFERROR(H6/G6,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J6" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A6,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I6=1,"✅ Completed",IF(I6&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="K6" s="10" t="s">
         <v>75</v>
@@ -10049,7 +10049,7 @@
       <c r="K28" s="10"/>
       <c r="L28" s="10"/>
       <c r="M28" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N28" s="10"/>
       <c r="O28" s="10" t="s">
@@ -10057,7 +10057,7 @@
       </c>
       <c r="P28" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M28)),1,IF(ISNUMBER(SEARCH("In Progress",M28)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="78.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Sync Project_Tracker.xlsx: VER-002 done, Sprint 5 complete
Marks VER-002 Done and refreshes every formula-driven rollup that
reads from it: Sprint 5, Milestone ML5, and Epic ML5-EP02 all now
show Completed (2 of 2 stories done); the Dashboard's current
milestone/sprint advance to ML6/SP06, upcoming sprint to SP07, and
completed-epic/story counts and overall progress percentage are
current. Applied via the same raw-XML cell patching used for every
prior sync, to avoid the conditional-formatting-dropping issue an
openpyxl round-trip causes on this workbook.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4370,7 +4370,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.34375</v>
+        <v>0.37083333333333335</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4389,7 +4389,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="0" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4421,7 +4421,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
@@ -4445,7 +4445,7 @@
         <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
@@ -4461,7 +4461,7 @@
         <v>28</v>
       </c>
       <c r="J10" s="0" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4493,7 +4493,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">COUNTA(Milestones!$B$2:$B$25)</f>
@@ -4517,7 +4517,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4541,7 +4541,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -4590,7 +4590,7 @@
         <v>36</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -4633,7 +4633,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B7</f>
-        <v>0.34375</v>
+        <v>0.37083333333333335</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
@@ -5388,7 +5388,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.375</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5757,11 +5757,11 @@
       <c r="I6" s="12"/>
       <c r="J6" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B6)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B6),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K6" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B6,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J6=1,"✅ Completed",IF(J6&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="L6" s="12" t="n">
         <v>0</v>
@@ -6630,11 +6630,11 @@
       <c r="I9" s="10"/>
       <c r="J9" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C9)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C9),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C9,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J9=1,"✅ Completed",IF(J9&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7831,15 +7831,15 @@
       </c>
       <c r="H6" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A6)*(Stories!$P$2:$P$200))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I6" s="11" t="n">
         <f aca="false">IFERROR(H6/G6,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J6" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A6,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I6=1,"✅ Completed",IF(I6&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="K6" s="10" t="s">
         <v>75</v>
@@ -10092,7 +10092,7 @@
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
       <c r="M29" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N29" s="10"/>
       <c r="O29" s="10" t="s">
@@ -10100,7 +10100,7 @@
       </c>
       <c r="P29" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M29)),1,IF(ISNUMBER(SEARCH("In Progress",M29)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="78.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
tracker: update hardcoded Completed Epics/Stories dashboard counters
Dashboard's Completed Phases/Milestones/Epics/Stories cells are
manually-maintained counters, not live formulas. DIR-001 completing
means Completed Epics goes 8->9 (ML6-EP01 is now fully done) and
Completed Stories goes 28->29 -- missed in the prior tracker commit.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4517,7 +4517,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4541,7 +4541,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>

</xml_diff>

<commit_message>
tracker: mark CTG-001 done, roll up Sprint 7/ML7/PH2/Dashboard progress
Stories: CTG-001 status flipped to Done. Rolled the change through
every dependent sheet: Epics (ML7-EP03 now 1/1, Completed),
Milestones (ML7 now 0.33, In Progress -- AI-001/AI-002 still
planned), Sprints (SP07 now 1/3, In Progress), Phase Tracker (PH2
now 0.538), and Dashboard's overall weighted progress (0.45) and
hardcoded Completed Epics/Stories counters (10/30).

Edited via the established raw-XML cell-patching method, verified
via openpyxl read-only/data_only that every rollup is internally
consistent, and via diff against the unzipped original that only
the six affected sheets changed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.4</v>
+        <v>0.44999999999999996</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">'Phase Tracker'!E3</f>
-        <v>0.46153846153846156</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="I9" s="0" t="s">
         <v>25</v>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.46153846153846156</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5853,11 +5853,11 @@
       <c r="I8" s="12"/>
       <c r="J8" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B8)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B8),0)</f>
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="K8" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B8,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J8=1,"✅ Completed",IF(J8&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="L8" s="12" t="n">
         <v>0</v>
@@ -7097,11 +7097,11 @@
       <c r="I24" s="10"/>
       <c r="J24" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C24)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C24),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C24,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J24=1,"✅ Completed",IF(J24&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7957,15 +7957,15 @@
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A8)*(Stories!$P$2:$P$200))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" s="11" t="n">
         <f aca="false">IFERROR(H8/G8,0)</f>
-        <v>0</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="J8" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A8,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I8=1,"✅ Completed",IF(I8&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>81</v>
@@ -10957,13 +10957,13 @@
       <c r="K48" s="10"/>
       <c r="L48" s="10"/>
       <c r="M48" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N48" s="10"/>
       <c r="O48" s="10"/>
       <c r="P48" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M48)),1,IF(ISNUMBER(SEARCH("In Progress",M48)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
tracker: mark CLM-001 done -- Sprint 6/ML6 fully complete
Stories: CLM-001 status flipped to Done. Rolled the change through
every dependent sheet: Epics (ML6-EP02 now 1/1, Completed),
Milestones (ML6 now 2/2, Completed), Sprints (SP06 now 2/2,
Completed), Phase Tracker (PH2 now 0.615), and Dashboard's overall
weighted progress (0.5) plus hardcoded Completed
Milestones/Epics/Stories counters (6/11/31).

Edited via the established raw-XML cell-patching method, verified
via openpyxl read-only/data_only that every rollup is internally
consistent, and via diff against the unzipped original that only
the six affected sheets changed.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.44999999999999996</v>
+        <v>0.5</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">'Phase Tracker'!E3</f>
-        <v>0.5384615384615384</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="I9" s="0" t="s">
         <v>25</v>
@@ -4525,7 +4525,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">COUNTA(Milestones!$B$2:$B$25)</f>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.5384615384615384</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5821,11 +5821,11 @@
       <c r="I7" s="12"/>
       <c r="J7" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B7)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B7),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K7" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B7,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J7=1,"✅ Completed",IF(J7&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="L7" s="12" t="n">
         <v>0</v>
@@ -6720,11 +6720,11 @@
       <c r="I11" s="10"/>
       <c r="J11" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C11)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C11),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C11,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J11=1,"✅ Completed",IF(J11&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7918,15 +7918,15 @@
       </c>
       <c r="H7" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A7)*(Stories!$P$2:$P$200))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I7" s="11" t="n">
         <f aca="false">IFERROR(H7/G7,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J7" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A7,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I7=1,"✅ Completed",IF(I7&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="K7" s="10" t="s">
         <v>78</v>
@@ -10226,7 +10226,7 @@
       <c r="K31" s="10"/>
       <c r="L31" s="10"/>
       <c r="M31" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N31" s="10"/>
       <c r="O31" s="10" t="s">
@@ -10234,7 +10234,7 @@
       </c>
       <c r="P31" s="10" t="n">
         <f aca="false">IF(ISNUMBER(SEARCH("Done",M31)),1,IF(ISNUMBER(SEARCH("In Progress",M31)),0.5,0))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="78.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
tracker: mark AI-001 done -- Epic ML7-EP01 complete, Sprint 7 2/3 done
AI-001 flipped to Done in Stories, propagated through Epic ML7-EP01
(now Completed, its only story), Milestone ML7 (2/3 stories done),
Sprint SP07 (2/3 done), Phase Tracker PH2, and the Dashboard.

Also corrected two stale cached rollups found while propagating: Phase
Tracker PH2's progress (grown from 13 to 25 stories since it was last
cached, now 14/25=0.56) and the Dashboard's Current Milestone/Current
Sprint/Upcoming Sprint pointers (still showing ML6/SP06/SP07 even
though Sprint 6 fully closed out with CLM-001 -- now ML7/SP07/SP08).

Dashboard: Overall Progress 0.464 (was showing a stale 0.5), Completed
Epics 12 (was 11), Completed Stories 32 (was 31).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.5</v>
+        <v>0.464</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">'Phase Tracker'!E3</f>
-        <v>0.6153846153846154</v>
+        <v>0.56</v>
       </c>
       <c r="I9" s="0" t="s">
         <v>25</v>
@@ -4477,7 +4477,7 @@
         <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -4622,7 +4622,7 @@
         <v>36</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -4665,7 +4665,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B7</f>
-        <v>0.37083333333333335</v>
+        <v>0.464</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.6153846153846154</v>
+        <v>0.56</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5853,7 +5853,7 @@
       <c r="I8" s="12"/>
       <c r="J8" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B8)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B8),0)</f>
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="K8" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B8,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J8=1,"✅ Completed",IF(J8&gt;0,"🔄 In Progress","⏳ Planned")))</f>
@@ -6749,11 +6749,11 @@
       <c r="I12" s="10"/>
       <c r="J12" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C12)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C12),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C12,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J12=1,"✅ Completed",IF(J12&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7957,11 +7957,11 @@
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A8)*(Stories!$P$2:$P$200))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I8" s="11" t="n">
         <f aca="false">IFERROR(H8/G8,0)</f>
-        <v>0.3333333333333333</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="J8" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A8,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I8=1,"✅ Completed",IF(I8&gt;0,"🔄 In Progress","⏳ Planned")))</f>
@@ -10269,7 +10269,7 @@
       <c r="K32" s="10"/>
       <c r="L32" s="10"/>
       <c r="M32" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N32" s="10"/>
       <c r="O32" s="10" t="s">

</xml_diff>

<commit_message>
tracker: mark AI-002 done -- Sprint 7 and Milestone ML7 fully complete
AI-002 flipped to Done, propagated through Epic ML7-EP02 (Completed,
its only story), Milestone ML7 (3/3 stories done -- Completed), Sprint
SP07 (3/3 done -- Completed), Phase Tracker PH2, and the Dashboard.

Dashboard: Overall Progress 0.49, Completed Milestones 7 (was 6),
Completed Epics 13 (was 12), Completed Stories 33 (was 32), Current
Milestone/Sprint advanced to ML8/SP08, Upcoming Sprint to SP09.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.464</v>
+        <v>0.49</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">'Phase Tracker'!E3</f>
-        <v>0.56</v>
+        <v>0.6</v>
       </c>
       <c r="I9" s="0" t="s">
         <v>25</v>
@@ -4477,7 +4477,7 @@
         <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
@@ -4525,7 +4525,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">COUNTA(Milestones!$B$2:$B$25)</f>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -4622,7 +4622,7 @@
         <v>36</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -4665,7 +4665,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B7</f>
-        <v>0.464</v>
+        <v>0.49</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.56</v>
+        <v>0.6</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5853,11 +5853,11 @@
       <c r="I8" s="12"/>
       <c r="J8" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B8)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B8),0)</f>
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="K8" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B8,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J8=1,"✅ Completed",IF(J8&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="L8" s="12" t="n">
         <v>0</v>
@@ -6778,11 +6778,11 @@
       <c r="I13" s="10"/>
       <c r="J13" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C13)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C13),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C13,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J13=1,"✅ Completed",IF(J13&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7957,15 +7957,15 @@
       </c>
       <c r="H8" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A8)*(Stories!$P$2:$P$200))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I8" s="11" t="n">
         <f aca="false">IFERROR(H8/G8,0)</f>
-        <v>0.6666666666666666</v>
+        <v>1</v>
       </c>
       <c r="J8" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A8,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I8=1,"✅ Completed",IF(I8&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="K8" s="10" t="s">
         <v>81</v>
@@ -10312,7 +10312,7 @@
       <c r="K33" s="10"/>
       <c r="L33" s="10"/>
       <c r="M33" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N33" s="10"/>
       <c r="O33" s="10" t="s">

</xml_diff>

<commit_message>
tracker: mark MAT-001 done -- Epic ML8-EP01 complete, Sprint 8 1/2 done
MAT-001 flipped to Done in Stories, propagated through Epic ML8-EP01
(now Completed, its only story), Milestone ML8 (1/2 stories done,
In Progress), Sprint SP08 (1/2 done, In Progress), Phase Tracker PH2,
and the Dashboard.

Dashboard: Overall Progress 0.516 (was 0.49), Completed Epics 14
(was 13), Completed Stories 34 (was 33). Current Milestone/Sprint
remain ML8/SP08 (not yet complete -- CON-001 is the remaining story).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.49</v>
+        <v>0.516</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">'Phase Tracker'!E3</f>
-        <v>0.6</v>
+        <v>0.64</v>
       </c>
       <c r="I9" s="0" t="s">
         <v>25</v>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -4665,7 +4665,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B7</f>
-        <v>0.49</v>
+        <v>0.516</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.6</v>
+        <v>0.64</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5885,11 +5885,11 @@
       <c r="I9" s="12"/>
       <c r="J9" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B9)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B9),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="K9" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B9,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J9=1,"✅ Completed",IF(J9&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="L9" s="12" t="n">
         <v>0</v>
@@ -6807,11 +6807,11 @@
       <c r="I14" s="10"/>
       <c r="J14" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C14)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C14),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C14,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J14=1,"✅ Completed",IF(J14&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7996,15 +7996,15 @@
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A9)*(Stories!$P$2:$P$200))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" s="11" t="n">
         <f aca="false">IFERROR(H9/G9,0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J9" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A9,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I9=1,"✅ Completed",IF(I9&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>🔄 In Progress</v>
       </c>
       <c r="K9" s="10" t="s">
         <v>84</v>
@@ -10355,7 +10355,7 @@
       <c r="K34" s="10"/>
       <c r="L34" s="10"/>
       <c r="M34" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N34" s="10"/>
       <c r="O34" s="10" t="s">

</xml_diff>

<commit_message>
tracker: mark CON-001 done -- Sprint 8 and Milestone ML8 fully complete
CON-001 flipped to Done, propagated through Epic ML8-EP02 (Completed,
its only story), Milestone ML8 (2/2 stories -- Completed), Sprint SP08
(2/2 -- Completed), Phase Tracker PH2, and the Dashboard.

Dashboard: Overall Progress 0.542 (was 0.516), Completed Milestones 8
(was 7), Completed Epics 15 (was 14), Completed Stories 35 (was 34).
Current Milestone/Sprint advanced to ML9/SP09, Upcoming Sprint to SP10.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MAg3bEPTDevTip5zp39mas
</commit_message>
<xml_diff>
--- a/docs/AI/Project_Tracker.xlsx
+++ b/docs/AI/Project_Tracker.xlsx
@@ -4402,7 +4402,7 @@
       </c>
       <c r="B7" s="6" t="n">
         <f aca="false">SUMPRODUCT('Phase Tracker'!$E$2:$E$7,'Phase Tracker'!$D$2:$D$7)</f>
-        <v>0.516</v>
+        <v>0.542</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
@@ -4453,7 +4453,7 @@
         <v>23</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
@@ -4463,7 +4463,7 @@
       </c>
       <c r="G9" s="7" t="n">
         <f aca="false">'Phase Tracker'!E3</f>
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="I9" s="0" t="s">
         <v>25</v>
@@ -4477,7 +4477,7 @@
         <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
@@ -4525,7 +4525,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" s="5" t="n">
         <f aca="false">COUNTA(Milestones!$B$2:$B$25)</f>
@@ -4549,7 +4549,7 @@
         <v>31</v>
       </c>
       <c r="B13" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="5" t="n">
         <f aca="false">COUNTA(Epics!$C$2:C$100)</f>
@@ -4573,7 +4573,7 @@
         <v>32</v>
       </c>
       <c r="B14" s="5" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C14" s="5" t="n">
         <f aca="false">B15</f>
@@ -4622,7 +4622,7 @@
         <v>36</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="C18" s="5"/>
       <c r="D18" s="5"/>
@@ -4665,7 +4665,7 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B7</f>
-        <v>0.516</v>
+        <v>0.542</v>
       </c>
       <c r="C21" s="6" t="n">
         <v>1</v>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="E3" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$E$2:$E$200=A3)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$E$2:$E$200,A3),0)</f>
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="F3" s="11" t="str">
         <f aca="false">IF(E3=1,"✅ Completed",IF(E3&gt;0,"🔄 In Progress","⏳ Planned"))</f>
@@ -5885,11 +5885,11 @@
       <c r="I9" s="12"/>
       <c r="J9" s="15" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$D$2:$D$200=B9)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$D$2:$D$200,B9),0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K9" s="12" t="str">
         <f aca="false">IF(COUNTIFS(Epics!$B$2:$B$100,B9,Epics!$K$2:$K$100,"*Blocked*")&gt;0,"🚫 Blocked",IF(J9=1,"✅ Completed",IF(J9&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="L9" s="12" t="n">
         <v>0</v>
@@ -6836,11 +6836,11 @@
       <c r="I15" s="10"/>
       <c r="J15" s="11" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Stories!$C$2:$C$200=C15)*(Stories!$P$2:$P$200))/COUNTIF(Stories!$C$2:$C$200,C15),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$C$2:$C$200,C15,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(J15=1,"✅ Completed",IF(J15&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>⏳ Planned</v>
+        <v>✅ Completed</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7996,15 +7996,15 @@
       </c>
       <c r="H9" s="10" t="n">
         <f aca="false">SUMPRODUCT((Stories!$B$2:$B$200=A9)*(Stories!$P$2:$P$200))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="11" t="n">
         <f aca="false">IFERROR(H9/G9,0)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="J9" s="11" t="str">
         <f aca="false">IF(COUNTIFS(Stories!$B$2:$B$200,A9,Stories!$M$2:$M$200,"*Blocked*")&gt;0,"🚫 Blocked",IF(I9=1,"✅ Completed",IF(I9&gt;0,"🔄 In Progress","⏳ Planned")))</f>
-        <v>🔄 In Progress</v>
+        <v>✅ Completed</v>
       </c>
       <c r="K9" s="10" t="s">
         <v>84</v>
@@ -10398,7 +10398,7 @@
       <c r="K35" s="10"/>
       <c r="L35" s="10"/>
       <c r="M35" s="10" t="s">
-        <v>296</v>
+        <v>19</v>
       </c>
       <c r="N35" s="10"/>
       <c r="O35" s="10" t="s">

</xml_diff>